<commit_message>
feat(import): support summary and period label in v2
</commit_message>
<xml_diff>
--- a/docs/catalog-import/catalog-import-v2-template.xlsx
+++ b/docs/catalog-import/catalog-import-v2-template.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="228">
   <si>
     <t>批次内关联 ID【必填】</t>
   </si>
@@ -33,6 +33,12 @@
     <t>类别【必填】</t>
   </si>
   <si>
+    <t>标题下导语</t>
+  </si>
+  <si>
+    <t>年代标签</t>
+  </si>
+  <si>
     <t>朝代</t>
   </si>
   <si>
@@ -129,6 +135,12 @@
     <t>catalogKind</t>
   </si>
   <si>
+    <t>summary</t>
+  </si>
+  <si>
+    <t>periodLabel</t>
+  </si>
+  <si>
     <t>dynasty</t>
   </si>
   <si>
@@ -309,10 +321,10 @@
     <t>4. 五个数据表都用 catalogImportId 关联 01_Catalog；catalogImportId ≠ sourceId ≠ catalogId。</t>
   </si>
   <si>
-    <t>5. value 有内容时，state 留空或选 VALUE；state 与 action 的英文 machine value 不翻译。</t>
-  </si>
-  <si>
-    <t>6. blank 或 UNSUPPLIED 表示本批次未提供；允许 UNKNOWN / NOT_APPLICABLE 的字段可用相应状态。</t>
+    <t>5. summary / periodLabel 是无 state 的直接可选文本；留空表示省略且不清除既有值。</t>
+  </si>
+  <si>
+    <t>6. 其余 value 有内容时，state 留空或选 VALUE；state 与 action 的英文 machine value 不翻译。blank 或 UNSUPPLIED 表示本批次未提供。</t>
   </si>
   <si>
     <t>7. CLEAR 才表示请求清除，并需要逐字段审批；blank ≠ delete。</t>
@@ -333,7 +345,7 @@
     <t>Identity：catalogImportId 是 batch-local 关联键；sourceId 是来源记录身份；catalogId 是 Catalog 身份。三者不可互换。CatalogId / SourceId linkage conflict 不可审批、不可 Apply。</t>
   </si>
   <si>
-    <t>State：一般事实字段与 scriptStyle 可用五种 state；description 与三个长文本字段仅用 VALUE / UNSUPPLIED / CLEAR。非 VALUE state 时 value 必须为空。</t>
+    <t>State：summary / periodLabel 没有 state 或 CLEAR；一般事实字段与 scriptStyle 可用五种 state；description 与三个长文本字段仅用 VALUE / UNSUPPLIED / CLEAR。非 VALUE state 时 value 必须为空。</t>
   </si>
   <si>
     <t>Location：province / prefecture / county 是行政区；currentLocation 是具体地点或遗址；currentCustodian 是当前管理或保管机构。</t>
@@ -423,6 +435,18 @@
     <t>选填</t>
   </si>
   <si>
+    <t>直接可选文本，最多 2,000 字符；留空会省略且不清除既有值，无 state / CLEAR 语义。</t>
+  </si>
+  <si>
+    <t>纯合成标题下导语</t>
+  </si>
+  <si>
+    <t>标题区展示的简短年代标签，最多 200 字符；留空会省略且不清除既有值，无 state / CLEAR 语义。</t>
+  </si>
+  <si>
+    <t>唐代（synthetic）</t>
+  </si>
+  <si>
     <t>原始事实文本；与右侧状态配对。</t>
   </si>
   <si>
@@ -645,7 +669,7 @@
     <t>D. Advanced persistence / approval / hash notes</t>
   </si>
   <si>
-    <t>V2 Apply 支持既有字段、四个内容字段、contributors 与 curated public citations；ownerNote 与既有 alias-update ambiguity 仍然 fail closed。</t>
+    <t>V2 Apply 支持 summary / periodLabel、既有字段、四个 stateful 内容字段、contributors 与 curated public citations；ownerNote 与既有 alias-update ambiguity 仍然 fail closed。</t>
   </si>
   <si>
     <t>PRESERVE 不改集合；REPLACE 以完整子表集合取代旧集合；CLEAR 删除完整集合。Create candidate 不允许 CLEAR。</t>
@@ -890,8 +914,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="CatalogImportTable" displayName="CatalogImportTable" ref="A2:AF3" totalsRowShown="1" headerRowCount="1">
-  <autoFilter ref="A2:AF3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="CatalogImportTable" displayName="CatalogImportTable" ref="A2:AH3" totalsRowShown="1" headerRowCount="1">
+  <autoFilter ref="A2:AH3">
     <filterColumn colId="0" hiddenButton="0"/>
     <filterColumn colId="1" hiddenButton="0"/>
     <filterColumn colId="2" hiddenButton="0"/>
@@ -924,40 +948,44 @@
     <filterColumn colId="29" hiddenButton="0"/>
     <filterColumn colId="30" hiddenButton="0"/>
     <filterColumn colId="31" hiddenButton="0"/>
+    <filterColumn colId="32" hiddenButton="0"/>
+    <filterColumn colId="33" hiddenButton="0"/>
   </autoFilter>
-  <tableColumns count="32">
+  <tableColumns count="34">
     <tableColumn id="1" name="catalogImportId" totalsRowLabel="Total"/>
     <tableColumn id="2" name="sourceId" totalsRowFunction="none"/>
     <tableColumn id="3" name="catalogId" totalsRowFunction="none"/>
     <tableColumn id="4" name="title" totalsRowFunction="none"/>
     <tableColumn id="5" name="catalogKind" totalsRowFunction="none"/>
-    <tableColumn id="6" name="dynasty" totalsRowFunction="none"/>
-    <tableColumn id="7" name="dynastyState" totalsRowFunction="none"/>
-    <tableColumn id="8" name="dateText" totalsRowFunction="none"/>
-    <tableColumn id="9" name="dateTextState" totalsRowFunction="none"/>
-    <tableColumn id="10" name="province" totalsRowFunction="none"/>
-    <tableColumn id="11" name="provinceState" totalsRowFunction="none"/>
-    <tableColumn id="12" name="prefecture" totalsRowFunction="none"/>
-    <tableColumn id="13" name="prefectureState" totalsRowFunction="none"/>
-    <tableColumn id="14" name="county" totalsRowFunction="none"/>
-    <tableColumn id="15" name="countyState" totalsRowFunction="none"/>
-    <tableColumn id="16" name="currentLocation" totalsRowFunction="none"/>
-    <tableColumn id="17" name="currentLocationState" totalsRowFunction="none"/>
-    <tableColumn id="18" name="currentCustodian" totalsRowFunction="none"/>
-    <tableColumn id="19" name="currentCustodianState" totalsRowFunction="none"/>
-    <tableColumn id="20" name="description" totalsRowFunction="none"/>
-    <tableColumn id="21" name="descriptionState" totalsRowFunction="none"/>
-    <tableColumn id="22" name="scriptStyle" totalsRowFunction="none"/>
-    <tableColumn id="23" name="scriptStyleState" totalsRowFunction="none"/>
-    <tableColumn id="24" name="transcription" totalsRowFunction="none"/>
-    <tableColumn id="25" name="transcriptionState" totalsRowFunction="none"/>
-    <tableColumn id="26" name="historicalContext" totalsRowFunction="none"/>
-    <tableColumn id="27" name="historicalContextState" totalsRowFunction="none"/>
-    <tableColumn id="28" name="scholarlyResearch" totalsRowFunction="none"/>
-    <tableColumn id="29" name="scholarlyResearchState" totalsRowFunction="none"/>
-    <tableColumn id="30" name="contributorsAction" totalsRowFunction="none"/>
-    <tableColumn id="31" name="publicCitationsAction" totalsRowFunction="none"/>
-    <tableColumn id="32" name="ownerNote" totalsRowFunction="none"/>
+    <tableColumn id="6" name="summary" totalsRowFunction="none"/>
+    <tableColumn id="7" name="periodLabel" totalsRowFunction="none"/>
+    <tableColumn id="8" name="dynasty" totalsRowFunction="none"/>
+    <tableColumn id="9" name="dynastyState" totalsRowFunction="none"/>
+    <tableColumn id="10" name="dateText" totalsRowFunction="none"/>
+    <tableColumn id="11" name="dateTextState" totalsRowFunction="none"/>
+    <tableColumn id="12" name="province" totalsRowFunction="none"/>
+    <tableColumn id="13" name="provinceState" totalsRowFunction="none"/>
+    <tableColumn id="14" name="prefecture" totalsRowFunction="none"/>
+    <tableColumn id="15" name="prefectureState" totalsRowFunction="none"/>
+    <tableColumn id="16" name="county" totalsRowFunction="none"/>
+    <tableColumn id="17" name="countyState" totalsRowFunction="none"/>
+    <tableColumn id="18" name="currentLocation" totalsRowFunction="none"/>
+    <tableColumn id="19" name="currentLocationState" totalsRowFunction="none"/>
+    <tableColumn id="20" name="currentCustodian" totalsRowFunction="none"/>
+    <tableColumn id="21" name="currentCustodianState" totalsRowFunction="none"/>
+    <tableColumn id="22" name="description" totalsRowFunction="none"/>
+    <tableColumn id="23" name="descriptionState" totalsRowFunction="none"/>
+    <tableColumn id="24" name="scriptStyle" totalsRowFunction="none"/>
+    <tableColumn id="25" name="scriptStyleState" totalsRowFunction="none"/>
+    <tableColumn id="26" name="transcription" totalsRowFunction="none"/>
+    <tableColumn id="27" name="transcriptionState" totalsRowFunction="none"/>
+    <tableColumn id="28" name="historicalContext" totalsRowFunction="none"/>
+    <tableColumn id="29" name="historicalContextState" totalsRowFunction="none"/>
+    <tableColumn id="30" name="scholarlyResearch" totalsRowFunction="none"/>
+    <tableColumn id="31" name="scholarlyResearchState" totalsRowFunction="none"/>
+    <tableColumn id="32" name="contributorsAction" totalsRowFunction="none"/>
+    <tableColumn id="33" name="publicCitationsAction" totalsRowFunction="none"/>
+    <tableColumn id="34" name="ownerNote" totalsRowFunction="none"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -1366,36 +1394,39 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AF3"/>
+  <dimension ref="A1:AH3"/>
   <sheetFormatPr defaultRowHeight="20" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
-    <col min="5" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="20" customWidth="1"/>
-    <col min="8" max="8" width="22" customWidth="1"/>
-    <col min="9" max="15" width="20" customWidth="1"/>
-    <col min="16" max="16" width="28" customWidth="1"/>
-    <col min="17" max="17" width="20" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="40" customWidth="1"/>
+    <col min="7" max="7" width="24" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="10" max="10" width="22" customWidth="1"/>
+    <col min="11" max="17" width="20" customWidth="1"/>
     <col min="18" max="18" width="28" customWidth="1"/>
     <col min="19" max="19" width="20" customWidth="1"/>
-    <col min="20" max="20" width="40" customWidth="1"/>
+    <col min="20" max="20" width="28" customWidth="1"/>
     <col min="21" max="21" width="20" customWidth="1"/>
-    <col min="22" max="22" width="28" customWidth="1"/>
+    <col min="22" max="22" width="40" customWidth="1"/>
     <col min="23" max="23" width="20" customWidth="1"/>
-    <col min="24" max="24" width="48" customWidth="1"/>
+    <col min="24" max="24" width="28" customWidth="1"/>
     <col min="25" max="25" width="20" customWidth="1"/>
-    <col min="26" max="26" width="42" customWidth="1"/>
+    <col min="26" max="26" width="48" customWidth="1"/>
     <col min="27" max="27" width="20" customWidth="1"/>
     <col min="28" max="28" width="42" customWidth="1"/>
     <col min="29" max="29" width="20" customWidth="1"/>
-    <col min="30" max="31" width="22" customWidth="1"/>
-    <col min="32" max="32" width="36" customWidth="1"/>
+    <col min="30" max="30" width="42" customWidth="1"/>
+    <col min="31" max="31" width="20" customWidth="1"/>
+    <col min="32" max="33" width="22" customWidth="1"/>
+    <col min="34" max="34" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="1" ht="34" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1414,7 +1445,7 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
@@ -1486,128 +1517,140 @@
       <c r="AD1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AE1" s="2" t="s">
         <v>30</v>
       </c>
       <c r="AF1" s="1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="2" ht="30" customHeight="1" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>40</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="O2" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Q2" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="S2" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="U2" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="W2" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="Y2" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="Z2" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="AA2" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="AB2" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="AC2" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="AD2" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="AE2" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
+      </c>
+      <c r="AE2" s="4" t="s">
+        <v>64</v>
       </c>
       <c r="AF2" s="3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="3" ht="24" customHeight="1" spans="1:32" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+      <c r="AG2" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="AH2" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
       <c r="D3" s="6"/>
       <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="7"/>
       <c r="I3" s="8"/>
-      <c r="J3" s="7"/>
+      <c r="J3" s="6"/>
       <c r="K3" s="8"/>
       <c r="L3" s="7"/>
       <c r="M3" s="8"/>
       <c r="N3" s="7"/>
       <c r="O3" s="8"/>
-      <c r="P3" s="6"/>
+      <c r="P3" s="7"/>
       <c r="Q3" s="8"/>
       <c r="R3" s="6"/>
       <c r="S3" s="8"/>
@@ -1621,9 +1664,11 @@
       <c r="AA3" s="8"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="8"/>
-      <c r="AD3" s="7"/>
-      <c r="AE3" s="7"/>
-      <c r="AF3" s="6"/>
+      <c r="AD3" s="6"/>
+      <c r="AE3" s="8"/>
+      <c r="AF3" s="7"/>
+      <c r="AG3" s="7"/>
+      <c r="AH3" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="15">
@@ -1633,17 +1678,17 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="长文本状态" prompt="有值时留空或选 VALUE；空值可选 UNSUPPLIED 或 CLEAR。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：VALUE / UNSUPPLIED / CLEAR" sqref="AC3:AC1048576">
       <formula1>"VALUE,UNSUPPLIED,CLEAR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="集合操作" prompt="留空等同 PRESERVE；仅选择 PRESERVE、REPLACE 或 CLEAR。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：PRESERVE / REPLACE / CLEAR" sqref="AD3:AD1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="长文本状态" prompt="有值时留空或选 VALUE；空值可选 UNSUPPLIED 或 CLEAR。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：VALUE / UNSUPPLIED / CLEAR" sqref="AE3:AE1048576">
+      <formula1>"VALUE,UNSUPPLIED,CLEAR"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="集合操作" prompt="留空等同 PRESERVE；仅选择 PRESERVE、REPLACE 或 CLEAR。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：PRESERVE / REPLACE / CLEAR" sqref="AF3:AF1048576">
       <formula1>"PRESERVE,REPLACE,CLEAR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="集合操作" prompt="留空等同 PRESERVE；仅选择 PRESERVE、REPLACE 或 CLEAR。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：PRESERVE / REPLACE / CLEAR" sqref="AE3:AE1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="集合操作" prompt="留空等同 PRESERVE；仅选择 PRESERVE、REPLACE 或 CLEAR。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：PRESERVE / REPLACE / CLEAR" sqref="AG3:AG1048576">
       <formula1>"PRESERVE,REPLACE,CLEAR"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="目录类型 / CatalogKind" prompt="请选择英文 machine value：inscription 或 calligraphy。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：inscription / calligraphy" sqref="E3:E1048576">
       <formula1>"inscription,calligraphy"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="事实字段状态" prompt="有值时留空或选 VALUE；空值可选 UNSUPPLIED、UNKNOWN、NOT_APPLICABLE 或 CLEAR。blank 不删除。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：VALUE / UNSUPPLIED / UNKNOWN / NOT_APPLICABLE / CLEAR" sqref="G3:G1048576">
-      <formula1>"VALUE,UNSUPPLIED,UNKNOWN,NOT_APPLICABLE,CLEAR"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="事实字段状态" prompt="有值时留空或选 VALUE；空值可选 UNSUPPLIED、UNKNOWN、NOT_APPLICABLE 或 CLEAR。blank 不删除。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：VALUE / UNSUPPLIED / UNKNOWN / NOT_APPLICABLE / CLEAR" sqref="I3:I1048576">
       <formula1>"VALUE,UNSUPPLIED,UNKNOWN,NOT_APPLICABLE,CLEAR"</formula1>
@@ -1663,14 +1708,14 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="事实字段状态" prompt="有值时留空或选 VALUE；空值可选 UNSUPPLIED、UNKNOWN、NOT_APPLICABLE 或 CLEAR。blank 不删除。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：VALUE / UNSUPPLIED / UNKNOWN / NOT_APPLICABLE / CLEAR" sqref="S3:S1048576">
       <formula1>"VALUE,UNSUPPLIED,UNKNOWN,NOT_APPLICABLE,CLEAR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="描述状态" prompt="有描述时留空或选 VALUE；空值可选 UNSUPPLIED 或 CLEAR。blank 不删除。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：VALUE / UNSUPPLIED / CLEAR" sqref="U3:U1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="事实字段状态" prompt="有值时留空或选 VALUE；空值可选 UNSUPPLIED、UNKNOWN、NOT_APPLICABLE 或 CLEAR。blank 不删除。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：VALUE / UNSUPPLIED / UNKNOWN / NOT_APPLICABLE / CLEAR" sqref="U3:U1048576">
+      <formula1>"VALUE,UNSUPPLIED,UNKNOWN,NOT_APPLICABLE,CLEAR"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="描述状态" prompt="有描述时留空或选 VALUE；空值可选 UNSUPPLIED 或 CLEAR。blank 不删除。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：VALUE / UNSUPPLIED / CLEAR" sqref="W3:W1048576">
       <formula1>"VALUE,UNSUPPLIED,CLEAR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="事实字段状态" prompt="有值时留空或选 VALUE；空值可选 UNSUPPLIED、UNKNOWN、NOT_APPLICABLE 或 CLEAR。blank 不删除。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：VALUE / UNSUPPLIED / UNKNOWN / NOT_APPLICABLE / CLEAR" sqref="W3:W1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="事实字段状态" prompt="有值时留空或选 VALUE；空值可选 UNSUPPLIED、UNKNOWN、NOT_APPLICABLE 或 CLEAR。blank 不删除。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：VALUE / UNSUPPLIED / UNKNOWN / NOT_APPLICABLE / CLEAR" sqref="Y3:Y1048576">
       <formula1>"VALUE,UNSUPPLIED,UNKNOWN,NOT_APPLICABLE,CLEAR"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="长文本状态" prompt="有值时留空或选 VALUE；空值可选 UNSUPPLIED 或 CLEAR。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：VALUE / UNSUPPLIED / CLEAR" sqref="Y3:Y1048576">
-      <formula1>"VALUE,UNSUPPLIED,CLEAR"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1699,21 +1744,21 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -1758,36 +1803,36 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -1826,27 +1871,27 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -1889,39 +1934,39 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -1943,7 +1988,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F93"/>
+  <dimension ref="A1:F95"/>
   <sheetFormatPr defaultRowHeight="20" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -1956,7 +2001,7 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -1966,7 +2011,7 @@
     </row>
     <row r="2" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -1976,7 +2021,7 @@
     </row>
     <row r="4" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B4" s="11"/>
       <c r="C4" s="11"/>
@@ -1986,7 +2031,7 @@
     </row>
     <row r="5" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B5" s="12"/>
       <c r="C5" s="12"/>
@@ -1996,7 +2041,7 @@
     </row>
     <row r="6" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B6" s="12"/>
       <c r="C6" s="12"/>
@@ -2006,7 +2051,7 @@
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B7" s="12"/>
       <c r="C7" s="12"/>
@@ -2016,7 +2061,7 @@
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B8" s="12"/>
       <c r="C8" s="12"/>
@@ -2026,7 +2071,7 @@
     </row>
     <row r="9" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12"/>
@@ -2036,7 +2081,7 @@
     </row>
     <row r="10" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B10" s="12"/>
       <c r="C10" s="12"/>
@@ -2046,7 +2091,7 @@
     </row>
     <row r="11" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12"/>
@@ -2056,7 +2101,7 @@
     </row>
     <row r="12" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B12" s="12"/>
       <c r="C12" s="12"/>
@@ -2066,7 +2111,7 @@
     </row>
     <row r="13" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12"/>
@@ -2076,7 +2121,7 @@
     </row>
     <row r="14" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B14" s="12"/>
       <c r="C14" s="12"/>
@@ -2086,7 +2131,7 @@
     </row>
     <row r="17" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
@@ -2096,7 +2141,7 @@
     </row>
     <row r="18" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12"/>
@@ -2106,7 +2151,7 @@
     </row>
     <row r="19" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B19" s="12"/>
       <c r="C19" s="12"/>
@@ -2116,7 +2161,7 @@
     </row>
     <row r="20" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B20" s="12"/>
       <c r="C20" s="12"/>
@@ -2126,7 +2171,7 @@
     </row>
     <row r="21" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B21" s="12"/>
       <c r="C21" s="12"/>
@@ -2136,7 +2181,7 @@
     </row>
     <row r="22" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B22" s="12"/>
       <c r="C22" s="12"/>
@@ -2146,7 +2191,7 @@
     </row>
     <row r="25" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B25" s="11"/>
       <c r="C25" s="11"/>
@@ -2156,1077 +2201,1097 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="13" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="F26" s="13" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="27" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E27" s="14" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F27" s="14" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="28" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E28" s="15" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="F28" s="15" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="29" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="F29" s="14" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="30" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E30" s="15" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="F30" s="15" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="31" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E31" s="14" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
     </row>
     <row r="32" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B32" s="15" t="s">
         <v>5</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E32" s="15" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="F32" s="15" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="33" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B33" s="14" t="s">
         <v>6</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="F33" s="14" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="34" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B34" s="15" t="s">
         <v>7</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E34" s="15" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="F34" s="15" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="35" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B35" s="14" t="s">
         <v>8</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E35" s="14" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="F35" s="14" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="36" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B36" s="15" t="s">
         <v>9</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E36" s="15" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="F36" s="15" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
     </row>
     <row r="37" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B37" s="14" t="s">
         <v>10</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E37" s="14" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="F37" s="14" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="38" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B38" s="15" t="s">
         <v>11</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D38" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E38" s="15" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="F38" s="15" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
     </row>
     <row r="39" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B39" s="14" t="s">
         <v>12</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D39" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E39" s="14" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="F39" s="14" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="40" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B40" s="15" t="s">
         <v>13</v>
       </c>
       <c r="C40" s="15" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D40" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E40" s="15" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="F40" s="15" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
     </row>
     <row r="41" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B41" s="14" t="s">
         <v>14</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D41" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E41" s="14" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="F41" s="14" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="42" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B42" s="15" t="s">
         <v>15</v>
       </c>
       <c r="C42" s="15" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D42" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E42" s="15" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="F42" s="15" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
     </row>
     <row r="43" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B43" s="14" t="s">
         <v>16</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D43" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E43" s="14" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="F43" s="14" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="44" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B44" s="15" t="s">
         <v>17</v>
       </c>
       <c r="C44" s="15" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D44" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E44" s="15" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="F44" s="15" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="45" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B45" s="14" t="s">
         <v>18</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D45" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E45" s="14" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="F45" s="14" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="46" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B46" s="15" t="s">
         <v>19</v>
       </c>
       <c r="C46" s="15" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D46" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E46" s="15" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="F46" s="15" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
     </row>
     <row r="47" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B47" s="14" t="s">
         <v>20</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D47" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E47" s="14" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="F47" s="14" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="48" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B48" s="15" t="s">
         <v>21</v>
       </c>
       <c r="C48" s="15" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D48" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E48" s="15" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="F48" s="15" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
     </row>
     <row r="49" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B49" s="14" t="s">
         <v>22</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D49" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E49" s="14" t="s">
-        <v>141</v>
+        <v>167</v>
       </c>
       <c r="F49" s="14" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="50" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B50" s="15" t="s">
         <v>23</v>
       </c>
       <c r="C50" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D50" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E50" s="15" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="F50" s="15" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
     </row>
     <row r="51" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B51" s="14" t="s">
         <v>24</v>
       </c>
       <c r="C51" s="14" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D51" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E51" s="14" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
       <c r="F51" s="14" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="52" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B52" s="15" t="s">
         <v>25</v>
       </c>
       <c r="C52" s="15" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D52" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E52" s="15" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="F52" s="15" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
     </row>
     <row r="53" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B53" s="14" t="s">
         <v>26</v>
       </c>
       <c r="C53" s="14" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D53" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E53" s="14" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="F53" s="14" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="54" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B54" s="15" t="s">
         <v>27</v>
       </c>
       <c r="C54" s="15" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D54" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E54" s="15" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="F54" s="15" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
     </row>
     <row r="55" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B55" s="14" t="s">
         <v>28</v>
       </c>
       <c r="C55" s="14" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D55" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E55" s="14" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="F55" s="14" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="56" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B56" s="15" t="s">
         <v>29</v>
       </c>
       <c r="C56" s="15" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D56" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E56" s="15" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="F56" s="15" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
     </row>
     <row r="57" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B57" s="14" t="s">
         <v>30</v>
       </c>
       <c r="C57" s="14" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D57" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E57" s="14" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="F57" s="14" t="s">
-        <v>168</v>
+        <v>146</v>
       </c>
     </row>
     <row r="58" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B58" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C58" s="15" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D58" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E58" s="15" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="F58" s="15" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
     </row>
     <row r="59" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="14" t="s">
-        <v>171</v>
+        <v>120</v>
       </c>
       <c r="B59" s="14" t="s">
-        <v>117</v>
+        <v>32</v>
       </c>
       <c r="C59" s="14" t="s">
-        <v>32</v>
+        <v>66</v>
       </c>
       <c r="D59" s="14" t="s">
-        <v>172</v>
+        <v>138</v>
       </c>
       <c r="E59" s="14" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F59" s="14" t="s">
-        <v>120</v>
+        <v>176</v>
       </c>
     </row>
     <row r="60" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="15" t="s">
-        <v>171</v>
+        <v>120</v>
       </c>
       <c r="B60" s="15" t="s">
-        <v>174</v>
+        <v>33</v>
       </c>
       <c r="C60" s="15" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D60" s="15" t="s">
-        <v>172</v>
+        <v>138</v>
       </c>
       <c r="E60" s="15" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="F60" s="15" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="61" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="14" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="B61" s="14" t="s">
-        <v>177</v>
+        <v>121</v>
       </c>
       <c r="C61" s="14" t="s">
-        <v>67</v>
+        <v>34</v>
       </c>
       <c r="D61" s="14" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="E61" s="14" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="F61" s="14" t="s">
-        <v>179</v>
+        <v>124</v>
       </c>
     </row>
     <row r="62" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="B62" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="C62" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="D62" s="15" t="s">
         <v>180</v>
       </c>
-      <c r="B62" s="15" t="s">
-        <v>117</v>
-      </c>
-      <c r="C62" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="D62" s="15" t="s">
-        <v>172</v>
-      </c>
       <c r="E62" s="15" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="F62" s="15" t="s">
-        <v>120</v>
+        <v>184</v>
       </c>
     </row>
     <row r="63" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="B63" s="14" t="s">
+        <v>185</v>
+      </c>
+      <c r="C63" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="D63" s="14" t="s">
         <v>180</v>
       </c>
-      <c r="B63" s="14" t="s">
-        <v>121</v>
-      </c>
-      <c r="C63" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="D63" s="14" t="s">
-        <v>172</v>
-      </c>
       <c r="E63" s="14" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="F63" s="14" t="s">
-        <v>123</v>
+        <v>187</v>
       </c>
     </row>
     <row r="64" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="15" t="s">
+        <v>188</v>
+      </c>
+      <c r="B64" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="C64" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="D64" s="15" t="s">
         <v>180</v>
       </c>
-      <c r="B64" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="C64" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="D64" s="15" t="s">
-        <v>134</v>
-      </c>
       <c r="E64" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F64" s="15" t="s">
-        <v>183</v>
+        <v>124</v>
       </c>
     </row>
     <row r="65" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="B65" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="C65" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="D65" s="14" t="s">
         <v>180</v>
       </c>
-      <c r="B65" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="C65" s="14" t="s">
-        <v>73</v>
-      </c>
-      <c r="D65" s="14" t="s">
-        <v>134</v>
-      </c>
       <c r="E65" s="14" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="F65" s="14" t="s">
-        <v>185</v>
+        <v>127</v>
       </c>
     </row>
     <row r="66" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="15" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="B66" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C66" s="15" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D66" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E66" s="15" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="F66" s="15" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
     </row>
     <row r="67" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="14" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="B67" s="14" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C67" s="14" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D67" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E67" s="14" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="F67" s="14" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
     </row>
     <row r="68" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="15" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B68" s="15" t="s">
-        <v>117</v>
+        <v>74</v>
       </c>
       <c r="C68" s="15" t="s">
-        <v>32</v>
+        <v>78</v>
       </c>
       <c r="D68" s="15" t="s">
-        <v>172</v>
+        <v>138</v>
       </c>
       <c r="E68" s="15" t="s">
-        <v>173</v>
+        <v>194</v>
       </c>
       <c r="F68" s="15" t="s">
-        <v>120</v>
+        <v>195</v>
       </c>
     </row>
     <row r="69" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="14" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B69" s="14" t="s">
-        <v>191</v>
+        <v>75</v>
       </c>
       <c r="C69" s="14" t="s">
         <v>79</v>
       </c>
       <c r="D69" s="14" t="s">
-        <v>172</v>
+        <v>138</v>
       </c>
       <c r="E69" s="14" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="F69" s="14" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
     </row>
     <row r="70" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="15" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="B70" s="15" t="s">
-        <v>194</v>
+        <v>121</v>
       </c>
       <c r="C70" s="15" t="s">
-        <v>80</v>
+        <v>34</v>
       </c>
       <c r="D70" s="15" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="E70" s="15" t="s">
-        <v>195</v>
+        <v>181</v>
       </c>
       <c r="F70" s="15" t="s">
-        <v>196</v>
+        <v>124</v>
       </c>
     </row>
     <row r="71" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="14" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="B71" s="14" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C71" s="14" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D71" s="14" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="E71" s="14" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F71" s="14" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="72" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="15" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B72" s="15" t="s">
-        <v>117</v>
+        <v>202</v>
       </c>
       <c r="C72" s="15" t="s">
-        <v>32</v>
+        <v>84</v>
       </c>
       <c r="D72" s="15" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="E72" s="15" t="s">
-        <v>173</v>
+        <v>203</v>
       </c>
       <c r="F72" s="15" t="s">
-        <v>120</v>
+        <v>204</v>
       </c>
     </row>
     <row r="73" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="14" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B73" s="14" t="s">
-        <v>191</v>
+        <v>205</v>
       </c>
       <c r="C73" s="14" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="D73" s="14" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="E73" s="14" t="s">
-        <v>192</v>
+        <v>206</v>
       </c>
       <c r="F73" s="14" t="s">
-        <v>193</v>
+        <v>207</v>
       </c>
     </row>
     <row r="74" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="15" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="B74" s="15" t="s">
-        <v>201</v>
+        <v>121</v>
       </c>
       <c r="C74" s="15" t="s">
-        <v>86</v>
+        <v>34</v>
       </c>
       <c r="D74" s="15" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="E74" s="15" t="s">
-        <v>202</v>
+        <v>181</v>
       </c>
       <c r="F74" s="15" t="s">
-        <v>183</v>
+        <v>124</v>
       </c>
     </row>
     <row r="75" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="14" t="s">
+        <v>208</v>
+      </c>
+      <c r="B75" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="C75" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="D75" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="E75" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="B75" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="C75" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="D75" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="E75" s="14" t="s">
-        <v>203</v>
-      </c>
       <c r="F75" s="14" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="76" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="15" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="B76" s="15" t="s">
-        <v>84</v>
+        <v>209</v>
       </c>
       <c r="C76" s="15" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D76" s="15" t="s">
-        <v>134</v>
+        <v>180</v>
       </c>
       <c r="E76" s="15" t="s">
-        <v>186</v>
+        <v>210</v>
       </c>
       <c r="F76" s="15" t="s">
-        <v>205</v>
+        <v>191</v>
       </c>
     </row>
     <row r="77" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="14" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="B77" s="14" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C77" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="D77" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="E77" s="14" t="s">
+        <v>211</v>
+      </c>
+      <c r="F77" s="14" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="78" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" s="15" t="s">
+        <v>208</v>
+      </c>
+      <c r="B78" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="C78" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="D78" s="15" t="s">
+        <v>138</v>
+      </c>
+      <c r="E78" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="F78" s="15" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="79" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" s="14" t="s">
+        <v>208</v>
+      </c>
+      <c r="B79" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="D77" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="E77" s="14" t="s">
-        <v>206</v>
-      </c>
-      <c r="F77" s="14" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="80" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A80" s="11" t="s">
-        <v>208</v>
-      </c>
-      <c r="B80" s="11"/>
-      <c r="C80" s="11"/>
-      <c r="D80" s="11"/>
-      <c r="E80" s="11"/>
-      <c r="F80" s="11"/>
-    </row>
-    <row r="81" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A81" s="12" t="s">
-        <v>209</v>
-      </c>
-      <c r="B81" s="12"/>
-      <c r="C81" s="12"/>
-      <c r="D81" s="12"/>
-      <c r="E81" s="12"/>
-      <c r="F81" s="12"/>
-    </row>
-    <row r="82" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A82" s="12" t="s">
-        <v>210</v>
-      </c>
-      <c r="B82" s="12"/>
-      <c r="C82" s="12"/>
-      <c r="D82" s="12"/>
-      <c r="E82" s="12"/>
-      <c r="F82" s="12"/>
+      <c r="C79" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="D79" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="E79" s="14" t="s">
+        <v>214</v>
+      </c>
+      <c r="F79" s="14" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="82" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" s="11" t="s">
+        <v>216</v>
+      </c>
+      <c r="B82" s="11"/>
+      <c r="C82" s="11"/>
+      <c r="D82" s="11"/>
+      <c r="E82" s="11"/>
+      <c r="F82" s="11"/>
     </row>
     <row r="83" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="12" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="B83" s="12"/>
       <c r="C83" s="12"/>
@@ -3236,7 +3301,7 @@
     </row>
     <row r="84" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="12" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="B84" s="12"/>
       <c r="C84" s="12"/>
@@ -3246,7 +3311,7 @@
     </row>
     <row r="85" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="12" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B85" s="12"/>
       <c r="C85" s="12"/>
@@ -3256,7 +3321,7 @@
     </row>
     <row r="86" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="12" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="B86" s="12"/>
       <c r="C86" s="12"/>
@@ -3264,25 +3329,45 @@
       <c r="E86" s="12"/>
       <c r="F86" s="12"/>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A91" s="16" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A92" s="17" t="s">
-        <v>216</v>
-      </c>
-      <c r="B92" s="17" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A93" s="17" t="s">
-        <v>218</v>
-      </c>
-      <c r="B93" s="17" t="s">
-        <v>219</v>
+    <row r="87" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="B87" s="12"/>
+      <c r="C87" s="12"/>
+      <c r="D87" s="12"/>
+      <c r="E87" s="12"/>
+      <c r="F87" s="12"/>
+    </row>
+    <row r="88" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="B88" s="12"/>
+      <c r="C88" s="12"/>
+      <c r="D88" s="12"/>
+      <c r="E88" s="12"/>
+      <c r="F88" s="12"/>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A93" s="16" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A94" s="17" t="s">
+        <v>224</v>
+      </c>
+      <c r="B94" s="17" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A95" s="17" t="s">
+        <v>226</v>
+      </c>
+      <c r="B95" s="17" t="s">
+        <v>227</v>
       </c>
     </row>
   </sheetData>
@@ -3307,13 +3392,13 @@
     <mergeCell ref="A21:F21"/>
     <mergeCell ref="A22:F22"/>
     <mergeCell ref="A25:F25"/>
-    <mergeCell ref="A80:F80"/>
-    <mergeCell ref="A81:F81"/>
     <mergeCell ref="A82:F82"/>
     <mergeCell ref="A83:F83"/>
     <mergeCell ref="A84:F84"/>
     <mergeCell ref="A85:F85"/>
     <mergeCell ref="A86:F86"/>
+    <mergeCell ref="A87:F87"/>
+    <mergeCell ref="A88:F88"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>

<commit_message>
feat(import): support summary and period label in v2 (#91)
Add bounded catalog-import/v2 support for optional summary and periodLabel fields, including approval policy, exact-layout template updates, persistence behavior, read precedence, and regression coverage.
</commit_message>
<xml_diff>
--- a/docs/catalog-import/catalog-import-v2-template.xlsx
+++ b/docs/catalog-import/catalog-import-v2-template.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="446" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="462" uniqueCount="228">
   <si>
     <t>批次内关联 ID【必填】</t>
   </si>
@@ -33,6 +33,12 @@
     <t>类别【必填】</t>
   </si>
   <si>
+    <t>标题下导语</t>
+  </si>
+  <si>
+    <t>年代标签</t>
+  </si>
+  <si>
     <t>朝代</t>
   </si>
   <si>
@@ -129,6 +135,12 @@
     <t>catalogKind</t>
   </si>
   <si>
+    <t>summary</t>
+  </si>
+  <si>
+    <t>periodLabel</t>
+  </si>
+  <si>
     <t>dynasty</t>
   </si>
   <si>
@@ -309,10 +321,10 @@
     <t>4. 五个数据表都用 catalogImportId 关联 01_Catalog；catalogImportId ≠ sourceId ≠ catalogId。</t>
   </si>
   <si>
-    <t>5. value 有内容时，state 留空或选 VALUE；state 与 action 的英文 machine value 不翻译。</t>
-  </si>
-  <si>
-    <t>6. blank 或 UNSUPPLIED 表示本批次未提供；允许 UNKNOWN / NOT_APPLICABLE 的字段可用相应状态。</t>
+    <t>5. summary / periodLabel 是无 state 的直接可选文本；留空表示省略且不清除既有值。</t>
+  </si>
+  <si>
+    <t>6. 其余 value 有内容时，state 留空或选 VALUE；state 与 action 的英文 machine value 不翻译。blank 或 UNSUPPLIED 表示本批次未提供。</t>
   </si>
   <si>
     <t>7. CLEAR 才表示请求清除，并需要逐字段审批；blank ≠ delete。</t>
@@ -333,7 +345,7 @@
     <t>Identity：catalogImportId 是 batch-local 关联键；sourceId 是来源记录身份；catalogId 是 Catalog 身份。三者不可互换。CatalogId / SourceId linkage conflict 不可审批、不可 Apply。</t>
   </si>
   <si>
-    <t>State：一般事实字段与 scriptStyle 可用五种 state；description 与三个长文本字段仅用 VALUE / UNSUPPLIED / CLEAR。非 VALUE state 时 value 必须为空。</t>
+    <t>State：summary / periodLabel 没有 state 或 CLEAR；一般事实字段与 scriptStyle 可用五种 state；description 与三个长文本字段仅用 VALUE / UNSUPPLIED / CLEAR。非 VALUE state 时 value 必须为空。</t>
   </si>
   <si>
     <t>Location：province / prefecture / county 是行政区；currentLocation 是具体地点或遗址；currentCustodian 是当前管理或保管机构。</t>
@@ -423,6 +435,18 @@
     <t>选填</t>
   </si>
   <si>
+    <t>直接可选文本，最多 2,000 字符；留空会省略且不清除既有值，无 state / CLEAR 语义。</t>
+  </si>
+  <si>
+    <t>纯合成标题下导语</t>
+  </si>
+  <si>
+    <t>标题区展示的简短年代标签，最多 200 字符；留空会省略且不清除既有值，无 state / CLEAR 语义。</t>
+  </si>
+  <si>
+    <t>唐代（synthetic）</t>
+  </si>
+  <si>
     <t>原始事实文本；与右侧状态配对。</t>
   </si>
   <si>
@@ -645,7 +669,7 @@
     <t>D. Advanced persistence / approval / hash notes</t>
   </si>
   <si>
-    <t>V2 Apply 支持既有字段、四个内容字段、contributors 与 curated public citations；ownerNote 与既有 alias-update ambiguity 仍然 fail closed。</t>
+    <t>V2 Apply 支持 summary / periodLabel、既有字段、四个 stateful 内容字段、contributors 与 curated public citations；ownerNote 与既有 alias-update ambiguity 仍然 fail closed。</t>
   </si>
   <si>
     <t>PRESERVE 不改集合；REPLACE 以完整子表集合取代旧集合；CLEAR 删除完整集合。Create candidate 不允许 CLEAR。</t>
@@ -890,8 +914,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="CatalogImportTable" displayName="CatalogImportTable" ref="A2:AF3" totalsRowShown="1" headerRowCount="1">
-  <autoFilter ref="A2:AF3">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="CatalogImportTable" displayName="CatalogImportTable" ref="A2:AH3" totalsRowShown="1" headerRowCount="1">
+  <autoFilter ref="A2:AH3">
     <filterColumn colId="0" hiddenButton="0"/>
     <filterColumn colId="1" hiddenButton="0"/>
     <filterColumn colId="2" hiddenButton="0"/>
@@ -924,40 +948,44 @@
     <filterColumn colId="29" hiddenButton="0"/>
     <filterColumn colId="30" hiddenButton="0"/>
     <filterColumn colId="31" hiddenButton="0"/>
+    <filterColumn colId="32" hiddenButton="0"/>
+    <filterColumn colId="33" hiddenButton="0"/>
   </autoFilter>
-  <tableColumns count="32">
+  <tableColumns count="34">
     <tableColumn id="1" name="catalogImportId" totalsRowLabel="Total"/>
     <tableColumn id="2" name="sourceId" totalsRowFunction="none"/>
     <tableColumn id="3" name="catalogId" totalsRowFunction="none"/>
     <tableColumn id="4" name="title" totalsRowFunction="none"/>
     <tableColumn id="5" name="catalogKind" totalsRowFunction="none"/>
-    <tableColumn id="6" name="dynasty" totalsRowFunction="none"/>
-    <tableColumn id="7" name="dynastyState" totalsRowFunction="none"/>
-    <tableColumn id="8" name="dateText" totalsRowFunction="none"/>
-    <tableColumn id="9" name="dateTextState" totalsRowFunction="none"/>
-    <tableColumn id="10" name="province" totalsRowFunction="none"/>
-    <tableColumn id="11" name="provinceState" totalsRowFunction="none"/>
-    <tableColumn id="12" name="prefecture" totalsRowFunction="none"/>
-    <tableColumn id="13" name="prefectureState" totalsRowFunction="none"/>
-    <tableColumn id="14" name="county" totalsRowFunction="none"/>
-    <tableColumn id="15" name="countyState" totalsRowFunction="none"/>
-    <tableColumn id="16" name="currentLocation" totalsRowFunction="none"/>
-    <tableColumn id="17" name="currentLocationState" totalsRowFunction="none"/>
-    <tableColumn id="18" name="currentCustodian" totalsRowFunction="none"/>
-    <tableColumn id="19" name="currentCustodianState" totalsRowFunction="none"/>
-    <tableColumn id="20" name="description" totalsRowFunction="none"/>
-    <tableColumn id="21" name="descriptionState" totalsRowFunction="none"/>
-    <tableColumn id="22" name="scriptStyle" totalsRowFunction="none"/>
-    <tableColumn id="23" name="scriptStyleState" totalsRowFunction="none"/>
-    <tableColumn id="24" name="transcription" totalsRowFunction="none"/>
-    <tableColumn id="25" name="transcriptionState" totalsRowFunction="none"/>
-    <tableColumn id="26" name="historicalContext" totalsRowFunction="none"/>
-    <tableColumn id="27" name="historicalContextState" totalsRowFunction="none"/>
-    <tableColumn id="28" name="scholarlyResearch" totalsRowFunction="none"/>
-    <tableColumn id="29" name="scholarlyResearchState" totalsRowFunction="none"/>
-    <tableColumn id="30" name="contributorsAction" totalsRowFunction="none"/>
-    <tableColumn id="31" name="publicCitationsAction" totalsRowFunction="none"/>
-    <tableColumn id="32" name="ownerNote" totalsRowFunction="none"/>
+    <tableColumn id="6" name="summary" totalsRowFunction="none"/>
+    <tableColumn id="7" name="periodLabel" totalsRowFunction="none"/>
+    <tableColumn id="8" name="dynasty" totalsRowFunction="none"/>
+    <tableColumn id="9" name="dynastyState" totalsRowFunction="none"/>
+    <tableColumn id="10" name="dateText" totalsRowFunction="none"/>
+    <tableColumn id="11" name="dateTextState" totalsRowFunction="none"/>
+    <tableColumn id="12" name="province" totalsRowFunction="none"/>
+    <tableColumn id="13" name="provinceState" totalsRowFunction="none"/>
+    <tableColumn id="14" name="prefecture" totalsRowFunction="none"/>
+    <tableColumn id="15" name="prefectureState" totalsRowFunction="none"/>
+    <tableColumn id="16" name="county" totalsRowFunction="none"/>
+    <tableColumn id="17" name="countyState" totalsRowFunction="none"/>
+    <tableColumn id="18" name="currentLocation" totalsRowFunction="none"/>
+    <tableColumn id="19" name="currentLocationState" totalsRowFunction="none"/>
+    <tableColumn id="20" name="currentCustodian" totalsRowFunction="none"/>
+    <tableColumn id="21" name="currentCustodianState" totalsRowFunction="none"/>
+    <tableColumn id="22" name="description" totalsRowFunction="none"/>
+    <tableColumn id="23" name="descriptionState" totalsRowFunction="none"/>
+    <tableColumn id="24" name="scriptStyle" totalsRowFunction="none"/>
+    <tableColumn id="25" name="scriptStyleState" totalsRowFunction="none"/>
+    <tableColumn id="26" name="transcription" totalsRowFunction="none"/>
+    <tableColumn id="27" name="transcriptionState" totalsRowFunction="none"/>
+    <tableColumn id="28" name="historicalContext" totalsRowFunction="none"/>
+    <tableColumn id="29" name="historicalContextState" totalsRowFunction="none"/>
+    <tableColumn id="30" name="scholarlyResearch" totalsRowFunction="none"/>
+    <tableColumn id="31" name="scholarlyResearchState" totalsRowFunction="none"/>
+    <tableColumn id="32" name="contributorsAction" totalsRowFunction="none"/>
+    <tableColumn id="33" name="publicCitationsAction" totalsRowFunction="none"/>
+    <tableColumn id="34" name="ownerNote" totalsRowFunction="none"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -1366,36 +1394,39 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AF3"/>
+  <dimension ref="A1:AH3"/>
   <sheetFormatPr defaultRowHeight="20" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="28" customWidth="1"/>
-    <col min="5" max="6" width="18" customWidth="1"/>
-    <col min="7" max="7" width="20" customWidth="1"/>
-    <col min="8" max="8" width="22" customWidth="1"/>
-    <col min="9" max="15" width="20" customWidth="1"/>
-    <col min="16" max="16" width="28" customWidth="1"/>
-    <col min="17" max="17" width="20" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="40" customWidth="1"/>
+    <col min="7" max="7" width="24" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="10" max="10" width="22" customWidth="1"/>
+    <col min="11" max="17" width="20" customWidth="1"/>
     <col min="18" max="18" width="28" customWidth="1"/>
     <col min="19" max="19" width="20" customWidth="1"/>
-    <col min="20" max="20" width="40" customWidth="1"/>
+    <col min="20" max="20" width="28" customWidth="1"/>
     <col min="21" max="21" width="20" customWidth="1"/>
-    <col min="22" max="22" width="28" customWidth="1"/>
+    <col min="22" max="22" width="40" customWidth="1"/>
     <col min="23" max="23" width="20" customWidth="1"/>
-    <col min="24" max="24" width="48" customWidth="1"/>
+    <col min="24" max="24" width="28" customWidth="1"/>
     <col min="25" max="25" width="20" customWidth="1"/>
-    <col min="26" max="26" width="42" customWidth="1"/>
+    <col min="26" max="26" width="48" customWidth="1"/>
     <col min="27" max="27" width="20" customWidth="1"/>
     <col min="28" max="28" width="42" customWidth="1"/>
     <col min="29" max="29" width="20" customWidth="1"/>
-    <col min="30" max="31" width="22" customWidth="1"/>
-    <col min="32" max="32" width="36" customWidth="1"/>
+    <col min="30" max="30" width="42" customWidth="1"/>
+    <col min="31" max="31" width="20" customWidth="1"/>
+    <col min="32" max="33" width="22" customWidth="1"/>
+    <col min="34" max="34" width="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" spans="1:32" x14ac:dyDescent="0.25">
+    <row r="1" ht="34" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1414,7 +1445,7 @@
       <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
@@ -1486,128 +1517,140 @@
       <c r="AD1" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AE1" s="2" t="s">
         <v>30</v>
       </c>
       <c r="AF1" s="1" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="2" ht="30" customHeight="1" spans="1:32" x14ac:dyDescent="0.25">
+      <c r="AG1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>40</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="K2" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="M2" s="4" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="N2" s="3" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="O2" s="4" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="P2" s="3" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="Q2" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="R2" s="3" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="S2" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="U2" s="4" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="V2" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="W2" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="Y2" s="4" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="Z2" s="3" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="AA2" s="4" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="AB2" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="AC2" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="AD2" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="AE2" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
+      </c>
+      <c r="AE2" s="4" t="s">
+        <v>64</v>
       </c>
       <c r="AF2" s="3" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="3" ht="24" customHeight="1" spans="1:32" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+      <c r="AG2" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="AH2" s="3" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" ht="24" customHeight="1" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A3" s="5"/>
       <c r="B3" s="5"/>
       <c r="C3" s="5"/>
       <c r="D3" s="6"/>
       <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+      <c r="H3" s="7"/>
       <c r="I3" s="8"/>
-      <c r="J3" s="7"/>
+      <c r="J3" s="6"/>
       <c r="K3" s="8"/>
       <c r="L3" s="7"/>
       <c r="M3" s="8"/>
       <c r="N3" s="7"/>
       <c r="O3" s="8"/>
-      <c r="P3" s="6"/>
+      <c r="P3" s="7"/>
       <c r="Q3" s="8"/>
       <c r="R3" s="6"/>
       <c r="S3" s="8"/>
@@ -1621,9 +1664,11 @@
       <c r="AA3" s="8"/>
       <c r="AB3" s="6"/>
       <c r="AC3" s="8"/>
-      <c r="AD3" s="7"/>
-      <c r="AE3" s="7"/>
-      <c r="AF3" s="6"/>
+      <c r="AD3" s="6"/>
+      <c r="AE3" s="8"/>
+      <c r="AF3" s="7"/>
+      <c r="AG3" s="7"/>
+      <c r="AH3" s="6"/>
     </row>
   </sheetData>
   <dataValidations count="15">
@@ -1633,17 +1678,17 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="长文本状态" prompt="有值时留空或选 VALUE；空值可选 UNSUPPLIED 或 CLEAR。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：VALUE / UNSUPPLIED / CLEAR" sqref="AC3:AC1048576">
       <formula1>"VALUE,UNSUPPLIED,CLEAR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="集合操作" prompt="留空等同 PRESERVE；仅选择 PRESERVE、REPLACE 或 CLEAR。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：PRESERVE / REPLACE / CLEAR" sqref="AD3:AD1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="长文本状态" prompt="有值时留空或选 VALUE；空值可选 UNSUPPLIED 或 CLEAR。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：VALUE / UNSUPPLIED / CLEAR" sqref="AE3:AE1048576">
+      <formula1>"VALUE,UNSUPPLIED,CLEAR"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="集合操作" prompt="留空等同 PRESERVE；仅选择 PRESERVE、REPLACE 或 CLEAR。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：PRESERVE / REPLACE / CLEAR" sqref="AF3:AF1048576">
       <formula1>"PRESERVE,REPLACE,CLEAR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="集合操作" prompt="留空等同 PRESERVE；仅选择 PRESERVE、REPLACE 或 CLEAR。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：PRESERVE / REPLACE / CLEAR" sqref="AE3:AE1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="集合操作" prompt="留空等同 PRESERVE；仅选择 PRESERVE、REPLACE 或 CLEAR。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：PRESERVE / REPLACE / CLEAR" sqref="AG3:AG1048576">
       <formula1>"PRESERVE,REPLACE,CLEAR"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="目录类型 / CatalogKind" prompt="请选择英文 machine value：inscription 或 calligraphy。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：inscription / calligraphy" sqref="E3:E1048576">
       <formula1>"inscription,calligraphy"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="事实字段状态" prompt="有值时留空或选 VALUE；空值可选 UNSUPPLIED、UNKNOWN、NOT_APPLICABLE 或 CLEAR。blank 不删除。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：VALUE / UNSUPPLIED / UNKNOWN / NOT_APPLICABLE / CLEAR" sqref="G3:G1048576">
-      <formula1>"VALUE,UNSUPPLIED,UNKNOWN,NOT_APPLICABLE,CLEAR"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="事实字段状态" prompt="有值时留空或选 VALUE；空值可选 UNSUPPLIED、UNKNOWN、NOT_APPLICABLE 或 CLEAR。blank 不删除。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：VALUE / UNSUPPLIED / UNKNOWN / NOT_APPLICABLE / CLEAR" sqref="I3:I1048576">
       <formula1>"VALUE,UNSUPPLIED,UNKNOWN,NOT_APPLICABLE,CLEAR"</formula1>
@@ -1663,14 +1708,14 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="事实字段状态" prompt="有值时留空或选 VALUE；空值可选 UNSUPPLIED、UNKNOWN、NOT_APPLICABLE 或 CLEAR。blank 不删除。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：VALUE / UNSUPPLIED / UNKNOWN / NOT_APPLICABLE / CLEAR" sqref="S3:S1048576">
       <formula1>"VALUE,UNSUPPLIED,UNKNOWN,NOT_APPLICABLE,CLEAR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="描述状态" prompt="有描述时留空或选 VALUE；空值可选 UNSUPPLIED 或 CLEAR。blank 不删除。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：VALUE / UNSUPPLIED / CLEAR" sqref="U3:U1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="事实字段状态" prompt="有值时留空或选 VALUE；空值可选 UNSUPPLIED、UNKNOWN、NOT_APPLICABLE 或 CLEAR。blank 不删除。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：VALUE / UNSUPPLIED / UNKNOWN / NOT_APPLICABLE / CLEAR" sqref="U3:U1048576">
+      <formula1>"VALUE,UNSUPPLIED,UNKNOWN,NOT_APPLICABLE,CLEAR"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="描述状态" prompt="有描述时留空或选 VALUE；空值可选 UNSUPPLIED 或 CLEAR。blank 不删除。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：VALUE / UNSUPPLIED / CLEAR" sqref="W3:W1048576">
       <formula1>"VALUE,UNSUPPLIED,CLEAR"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="事实字段状态" prompt="有值时留空或选 VALUE；空值可选 UNSUPPLIED、UNKNOWN、NOT_APPLICABLE 或 CLEAR。blank 不删除。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：VALUE / UNSUPPLIED / UNKNOWN / NOT_APPLICABLE / CLEAR" sqref="W3:W1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="事实字段状态" prompt="有值时留空或选 VALUE；空值可选 UNSUPPLIED、UNKNOWN、NOT_APPLICABLE 或 CLEAR。blank 不删除。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：VALUE / UNSUPPLIED / UNKNOWN / NOT_APPLICABLE / CLEAR" sqref="Y3:Y1048576">
       <formula1>"VALUE,UNSUPPLIED,UNKNOWN,NOT_APPLICABLE,CLEAR"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" promptTitle="长文本状态" prompt="有值时留空或选 VALUE；空值可选 UNSUPPLIED 或 CLEAR。" showErrorMessage="1" errorStyle="stop" errorTitle="值不符合 catalog-import/v2" error="请从下拉清单选择：VALUE / UNSUPPLIED / CLEAR" sqref="Y3:Y1048576">
-      <formula1>"VALUE,UNSUPPLIED,CLEAR"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1699,21 +1744,21 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
@@ -1758,36 +1803,36 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -1826,27 +1871,27 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -1889,39 +1934,39 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
     </row>
     <row r="3" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -1943,7 +1988,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F93"/>
+  <dimension ref="A1:F95"/>
   <sheetFormatPr defaultRowHeight="20" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="25" customWidth="1"/>
@@ -1956,7 +2001,7 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="9" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="B1" s="9"/>
       <c r="C1" s="9"/>
@@ -1966,7 +2011,7 @@
     </row>
     <row r="2" ht="34" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B2" s="10"/>
       <c r="C2" s="10"/>
@@ -1976,7 +2021,7 @@
     </row>
     <row r="4" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="11" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B4" s="11"/>
       <c r="C4" s="11"/>
@@ -1986,7 +2031,7 @@
     </row>
     <row r="5" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="12" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B5" s="12"/>
       <c r="C5" s="12"/>
@@ -1996,7 +2041,7 @@
     </row>
     <row r="6" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="12" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B6" s="12"/>
       <c r="C6" s="12"/>
@@ -2006,7 +2051,7 @@
     </row>
     <row r="7" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="12" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B7" s="12"/>
       <c r="C7" s="12"/>
@@ -2016,7 +2061,7 @@
     </row>
     <row r="8" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="12" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="B8" s="12"/>
       <c r="C8" s="12"/>
@@ -2026,7 +2071,7 @@
     </row>
     <row r="9" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="12" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B9" s="12"/>
       <c r="C9" s="12"/>
@@ -2036,7 +2081,7 @@
     </row>
     <row r="10" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="12" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B10" s="12"/>
       <c r="C10" s="12"/>
@@ -2046,7 +2091,7 @@
     </row>
     <row r="11" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="12" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="B11" s="12"/>
       <c r="C11" s="12"/>
@@ -2056,7 +2101,7 @@
     </row>
     <row r="12" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="12" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B12" s="12"/>
       <c r="C12" s="12"/>
@@ -2066,7 +2111,7 @@
     </row>
     <row r="13" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="12" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12"/>
@@ -2076,7 +2121,7 @@
     </row>
     <row r="14" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="12" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B14" s="12"/>
       <c r="C14" s="12"/>
@@ -2086,7 +2131,7 @@
     </row>
     <row r="17" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" s="11" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
@@ -2096,7 +2141,7 @@
     </row>
     <row r="18" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" s="12" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B18" s="12"/>
       <c r="C18" s="12"/>
@@ -2106,7 +2151,7 @@
     </row>
     <row r="19" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" s="12" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="B19" s="12"/>
       <c r="C19" s="12"/>
@@ -2116,7 +2161,7 @@
     </row>
     <row r="20" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B20" s="12"/>
       <c r="C20" s="12"/>
@@ -2126,7 +2171,7 @@
     </row>
     <row r="21" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B21" s="12"/>
       <c r="C21" s="12"/>
@@ -2136,7 +2181,7 @@
     </row>
     <row r="22" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B22" s="12"/>
       <c r="C22" s="12"/>
@@ -2146,7 +2191,7 @@
     </row>
     <row r="25" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25" s="11" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B25" s="11"/>
       <c r="C25" s="11"/>
@@ -2156,1077 +2201,1097 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26" s="13" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="B26" s="13" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="C26" s="13" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="D26" s="13" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="E26" s="13" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="F26" s="13" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
     </row>
     <row r="27" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D27" s="14" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E27" s="14" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="F27" s="14" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
     </row>
     <row r="28" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B28" s="15" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E28" s="15" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="F28" s="15" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="29" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B29" s="14" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="D29" s="14" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="E29" s="14" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="F29" s="14" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
     </row>
     <row r="30" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B30" s="15" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D30" s="15" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E30" s="15" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="F30" s="15" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
     </row>
     <row r="31" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D31" s="14" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="E31" s="14" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
     </row>
     <row r="32" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B32" s="15" t="s">
         <v>5</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E32" s="15" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="F32" s="15" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
     </row>
     <row r="33" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B33" s="14" t="s">
         <v>6</v>
       </c>
       <c r="C33" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D33" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E33" s="14" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="F33" s="14" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
     </row>
     <row r="34" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B34" s="15" t="s">
         <v>7</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E34" s="15" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="F34" s="15" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
     </row>
     <row r="35" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B35" s="14" t="s">
         <v>8</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D35" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E35" s="14" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="F35" s="14" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="36" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B36" s="15" t="s">
         <v>9</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E36" s="15" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="F36" s="15" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
     </row>
     <row r="37" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B37" s="14" t="s">
         <v>10</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D37" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E37" s="14" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="F37" s="14" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="38" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B38" s="15" t="s">
         <v>11</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D38" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E38" s="15" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="F38" s="15" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
     </row>
     <row r="39" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B39" s="14" t="s">
         <v>12</v>
       </c>
       <c r="C39" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D39" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E39" s="14" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="F39" s="14" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="40" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B40" s="15" t="s">
         <v>13</v>
       </c>
       <c r="C40" s="15" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D40" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E40" s="15" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="F40" s="15" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
     </row>
     <row r="41" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B41" s="14" t="s">
         <v>14</v>
       </c>
       <c r="C41" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D41" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E41" s="14" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="F41" s="14" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="42" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B42" s="15" t="s">
         <v>15</v>
       </c>
       <c r="C42" s="15" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D42" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E42" s="15" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="F42" s="15" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
     </row>
     <row r="43" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B43" s="14" t="s">
         <v>16</v>
       </c>
       <c r="C43" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D43" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E43" s="14" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="F43" s="14" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="44" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B44" s="15" t="s">
         <v>17</v>
       </c>
       <c r="C44" s="15" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D44" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E44" s="15" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="F44" s="15" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
     <row r="45" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B45" s="14" t="s">
         <v>18</v>
       </c>
       <c r="C45" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D45" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E45" s="14" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="F45" s="14" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="46" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B46" s="15" t="s">
         <v>19</v>
       </c>
       <c r="C46" s="15" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D46" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E46" s="15" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="F46" s="15" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
     </row>
     <row r="47" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B47" s="14" t="s">
         <v>20</v>
       </c>
       <c r="C47" s="14" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D47" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E47" s="14" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="F47" s="14" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="48" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B48" s="15" t="s">
         <v>21</v>
       </c>
       <c r="C48" s="15" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D48" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E48" s="15" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="F48" s="15" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
     </row>
     <row r="49" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B49" s="14" t="s">
         <v>22</v>
       </c>
       <c r="C49" s="14" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D49" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E49" s="14" t="s">
-        <v>141</v>
+        <v>167</v>
       </c>
       <c r="F49" s="14" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="50" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B50" s="15" t="s">
         <v>23</v>
       </c>
       <c r="C50" s="15" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="D50" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E50" s="15" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="F50" s="15" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
     </row>
     <row r="51" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B51" s="14" t="s">
         <v>24</v>
       </c>
       <c r="C51" s="14" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D51" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E51" s="14" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
       <c r="F51" s="14" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="52" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B52" s="15" t="s">
         <v>25</v>
       </c>
       <c r="C52" s="15" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="D52" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E52" s="15" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="F52" s="15" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
     </row>
     <row r="53" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B53" s="14" t="s">
         <v>26</v>
       </c>
       <c r="C53" s="14" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D53" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E53" s="14" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="F53" s="14" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="54" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B54" s="15" t="s">
         <v>27</v>
       </c>
       <c r="C54" s="15" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="D54" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E54" s="15" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="F54" s="15" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
     </row>
     <row r="55" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B55" s="14" t="s">
         <v>28</v>
       </c>
       <c r="C55" s="14" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D55" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E55" s="14" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="F55" s="14" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
     </row>
     <row r="56" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B56" s="15" t="s">
         <v>29</v>
       </c>
       <c r="C56" s="15" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D56" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E56" s="15" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="F56" s="15" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
     </row>
     <row r="57" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57" s="14" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B57" s="14" t="s">
         <v>30</v>
       </c>
       <c r="C57" s="14" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D57" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E57" s="14" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="F57" s="14" t="s">
-        <v>168</v>
+        <v>146</v>
       </c>
     </row>
     <row r="58" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" s="15" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B58" s="15" t="s">
         <v>31</v>
       </c>
       <c r="C58" s="15" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D58" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E58" s="15" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="F58" s="15" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
     </row>
     <row r="59" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" s="14" t="s">
-        <v>171</v>
+        <v>120</v>
       </c>
       <c r="B59" s="14" t="s">
-        <v>117</v>
+        <v>32</v>
       </c>
       <c r="C59" s="14" t="s">
-        <v>32</v>
+        <v>66</v>
       </c>
       <c r="D59" s="14" t="s">
-        <v>172</v>
+        <v>138</v>
       </c>
       <c r="E59" s="14" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F59" s="14" t="s">
-        <v>120</v>
+        <v>176</v>
       </c>
     </row>
     <row r="60" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60" s="15" t="s">
-        <v>171</v>
+        <v>120</v>
       </c>
       <c r="B60" s="15" t="s">
-        <v>174</v>
+        <v>33</v>
       </c>
       <c r="C60" s="15" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D60" s="15" t="s">
-        <v>172</v>
+        <v>138</v>
       </c>
       <c r="E60" s="15" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="F60" s="15" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
     </row>
     <row r="61" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61" s="14" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="B61" s="14" t="s">
-        <v>177</v>
+        <v>121</v>
       </c>
       <c r="C61" s="14" t="s">
-        <v>67</v>
+        <v>34</v>
       </c>
       <c r="D61" s="14" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="E61" s="14" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="F61" s="14" t="s">
-        <v>179</v>
+        <v>124</v>
       </c>
     </row>
     <row r="62" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="B62" s="15" t="s">
+        <v>182</v>
+      </c>
+      <c r="C62" s="15" t="s">
+        <v>70</v>
+      </c>
+      <c r="D62" s="15" t="s">
         <v>180</v>
       </c>
-      <c r="B62" s="15" t="s">
-        <v>117</v>
-      </c>
-      <c r="C62" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="D62" s="15" t="s">
-        <v>172</v>
-      </c>
       <c r="E62" s="15" t="s">
-        <v>173</v>
+        <v>183</v>
       </c>
       <c r="F62" s="15" t="s">
-        <v>120</v>
+        <v>184</v>
       </c>
     </row>
     <row r="63" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A63" s="14" t="s">
+        <v>179</v>
+      </c>
+      <c r="B63" s="14" t="s">
+        <v>185</v>
+      </c>
+      <c r="C63" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="D63" s="14" t="s">
         <v>180</v>
       </c>
-      <c r="B63" s="14" t="s">
-        <v>121</v>
-      </c>
-      <c r="C63" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="D63" s="14" t="s">
-        <v>172</v>
-      </c>
       <c r="E63" s="14" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="F63" s="14" t="s">
-        <v>123</v>
+        <v>187</v>
       </c>
     </row>
     <row r="64" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64" s="15" t="s">
+        <v>188</v>
+      </c>
+      <c r="B64" s="15" t="s">
+        <v>121</v>
+      </c>
+      <c r="C64" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="D64" s="15" t="s">
         <v>180</v>
       </c>
-      <c r="B64" s="15" t="s">
-        <v>68</v>
-      </c>
-      <c r="C64" s="15" t="s">
-        <v>72</v>
-      </c>
-      <c r="D64" s="15" t="s">
-        <v>134</v>
-      </c>
       <c r="E64" s="15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="F64" s="15" t="s">
-        <v>183</v>
+        <v>124</v>
       </c>
     </row>
     <row r="65" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65" s="14" t="s">
+        <v>188</v>
+      </c>
+      <c r="B65" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="C65" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="D65" s="14" t="s">
         <v>180</v>
       </c>
-      <c r="B65" s="14" t="s">
-        <v>69</v>
-      </c>
-      <c r="C65" s="14" t="s">
-        <v>73</v>
-      </c>
-      <c r="D65" s="14" t="s">
-        <v>134</v>
-      </c>
       <c r="E65" s="14" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="F65" s="14" t="s">
-        <v>185</v>
+        <v>127</v>
       </c>
     </row>
     <row r="66" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66" s="15" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="B66" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C66" s="15" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D66" s="15" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E66" s="15" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="F66" s="15" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
     </row>
     <row r="67" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67" s="14" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="B67" s="14" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C67" s="14" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D67" s="14" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="E67" s="14" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="F67" s="14" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
     </row>
     <row r="68" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68" s="15" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B68" s="15" t="s">
-        <v>117</v>
+        <v>74</v>
       </c>
       <c r="C68" s="15" t="s">
-        <v>32</v>
+        <v>78</v>
       </c>
       <c r="D68" s="15" t="s">
-        <v>172</v>
+        <v>138</v>
       </c>
       <c r="E68" s="15" t="s">
-        <v>173</v>
+        <v>194</v>
       </c>
       <c r="F68" s="15" t="s">
-        <v>120</v>
+        <v>195</v>
       </c>
     </row>
     <row r="69" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69" s="14" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B69" s="14" t="s">
-        <v>191</v>
+        <v>75</v>
       </c>
       <c r="C69" s="14" t="s">
         <v>79</v>
       </c>
       <c r="D69" s="14" t="s">
-        <v>172</v>
+        <v>138</v>
       </c>
       <c r="E69" s="14" t="s">
-        <v>192</v>
+        <v>196</v>
       </c>
       <c r="F69" s="14" t="s">
-        <v>193</v>
+        <v>197</v>
       </c>
     </row>
     <row r="70" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70" s="15" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="B70" s="15" t="s">
-        <v>194</v>
+        <v>121</v>
       </c>
       <c r="C70" s="15" t="s">
-        <v>80</v>
+        <v>34</v>
       </c>
       <c r="D70" s="15" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="E70" s="15" t="s">
-        <v>195</v>
+        <v>181</v>
       </c>
       <c r="F70" s="15" t="s">
-        <v>196</v>
+        <v>124</v>
       </c>
     </row>
     <row r="71" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71" s="14" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="B71" s="14" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="C71" s="14" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D71" s="14" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="E71" s="14" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F71" s="14" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="72" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72" s="15" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B72" s="15" t="s">
-        <v>117</v>
+        <v>202</v>
       </c>
       <c r="C72" s="15" t="s">
-        <v>32</v>
+        <v>84</v>
       </c>
       <c r="D72" s="15" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="E72" s="15" t="s">
-        <v>173</v>
+        <v>203</v>
       </c>
       <c r="F72" s="15" t="s">
-        <v>120</v>
+        <v>204</v>
       </c>
     </row>
     <row r="73" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73" s="14" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B73" s="14" t="s">
-        <v>191</v>
+        <v>205</v>
       </c>
       <c r="C73" s="14" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="D73" s="14" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="E73" s="14" t="s">
-        <v>192</v>
+        <v>206</v>
       </c>
       <c r="F73" s="14" t="s">
-        <v>193</v>
+        <v>207</v>
       </c>
     </row>
     <row r="74" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74" s="15" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="B74" s="15" t="s">
-        <v>201</v>
+        <v>121</v>
       </c>
       <c r="C74" s="15" t="s">
-        <v>86</v>
+        <v>34</v>
       </c>
       <c r="D74" s="15" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="E74" s="15" t="s">
-        <v>202</v>
+        <v>181</v>
       </c>
       <c r="F74" s="15" t="s">
-        <v>183</v>
+        <v>124</v>
       </c>
     </row>
     <row r="75" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75" s="14" t="s">
+        <v>208</v>
+      </c>
+      <c r="B75" s="14" t="s">
+        <v>199</v>
+      </c>
+      <c r="C75" s="14" t="s">
+        <v>83</v>
+      </c>
+      <c r="D75" s="14" t="s">
+        <v>180</v>
+      </c>
+      <c r="E75" s="14" t="s">
         <v>200</v>
       </c>
-      <c r="B75" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="C75" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="D75" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="E75" s="14" t="s">
-        <v>203</v>
-      </c>
       <c r="F75" s="14" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="76" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76" s="15" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="B76" s="15" t="s">
-        <v>84</v>
+        <v>209</v>
       </c>
       <c r="C76" s="15" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D76" s="15" t="s">
-        <v>134</v>
+        <v>180</v>
       </c>
       <c r="E76" s="15" t="s">
-        <v>186</v>
+        <v>210</v>
       </c>
       <c r="F76" s="15" t="s">
-        <v>205</v>
+        <v>191</v>
       </c>
     </row>
     <row r="77" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77" s="14" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="B77" s="14" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C77" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="D77" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="E77" s="14" t="s">
+        <v>211</v>
+      </c>
+      <c r="F77" s="14" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="78" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A78" s="15" t="s">
+        <v>208</v>
+      </c>
+      <c r="B78" s="15" t="s">
+        <v>88</v>
+      </c>
+      <c r="C78" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="D78" s="15" t="s">
+        <v>138</v>
+      </c>
+      <c r="E78" s="15" t="s">
+        <v>194</v>
+      </c>
+      <c r="F78" s="15" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="79" ht="32" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A79" s="14" t="s">
+        <v>208</v>
+      </c>
+      <c r="B79" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="D77" s="14" t="s">
-        <v>134</v>
-      </c>
-      <c r="E77" s="14" t="s">
-        <v>206</v>
-      </c>
-      <c r="F77" s="14" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="80" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A80" s="11" t="s">
-        <v>208</v>
-      </c>
-      <c r="B80" s="11"/>
-      <c r="C80" s="11"/>
-      <c r="D80" s="11"/>
-      <c r="E80" s="11"/>
-      <c r="F80" s="11"/>
-    </row>
-    <row r="81" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A81" s="12" t="s">
-        <v>209</v>
-      </c>
-      <c r="B81" s="12"/>
-      <c r="C81" s="12"/>
-      <c r="D81" s="12"/>
-      <c r="E81" s="12"/>
-      <c r="F81" s="12"/>
-    </row>
-    <row r="82" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A82" s="12" t="s">
-        <v>210</v>
-      </c>
-      <c r="B82" s="12"/>
-      <c r="C82" s="12"/>
-      <c r="D82" s="12"/>
-      <c r="E82" s="12"/>
-      <c r="F82" s="12"/>
+      <c r="C79" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="D79" s="14" t="s">
+        <v>138</v>
+      </c>
+      <c r="E79" s="14" t="s">
+        <v>214</v>
+      </c>
+      <c r="F79" s="14" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="82" ht="24" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A82" s="11" t="s">
+        <v>216</v>
+      </c>
+      <c r="B82" s="11"/>
+      <c r="C82" s="11"/>
+      <c r="D82" s="11"/>
+      <c r="E82" s="11"/>
+      <c r="F82" s="11"/>
     </row>
     <row r="83" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83" s="12" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="B83" s="12"/>
       <c r="C83" s="12"/>
@@ -3236,7 +3301,7 @@
     </row>
     <row r="84" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84" s="12" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="B84" s="12"/>
       <c r="C84" s="12"/>
@@ -3246,7 +3311,7 @@
     </row>
     <row r="85" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" s="12" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="B85" s="12"/>
       <c r="C85" s="12"/>
@@ -3256,7 +3321,7 @@
     </row>
     <row r="86" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" s="12" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="B86" s="12"/>
       <c r="C86" s="12"/>
@@ -3264,25 +3329,45 @@
       <c r="E86" s="12"/>
       <c r="F86" s="12"/>
     </row>
-    <row r="91" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A91" s="16" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A92" s="17" t="s">
-        <v>216</v>
-      </c>
-      <c r="B92" s="17" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A93" s="17" t="s">
-        <v>218</v>
-      </c>
-      <c r="B93" s="17" t="s">
-        <v>219</v>
+    <row r="87" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A87" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="B87" s="12"/>
+      <c r="C87" s="12"/>
+      <c r="D87" s="12"/>
+      <c r="E87" s="12"/>
+      <c r="F87" s="12"/>
+    </row>
+    <row r="88" ht="28" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A88" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="B88" s="12"/>
+      <c r="C88" s="12"/>
+      <c r="D88" s="12"/>
+      <c r="E88" s="12"/>
+      <c r="F88" s="12"/>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A93" s="16" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A94" s="17" t="s">
+        <v>224</v>
+      </c>
+      <c r="B94" s="17" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A95" s="17" t="s">
+        <v>226</v>
+      </c>
+      <c r="B95" s="17" t="s">
+        <v>227</v>
       </c>
     </row>
   </sheetData>
@@ -3307,13 +3392,13 @@
     <mergeCell ref="A21:F21"/>
     <mergeCell ref="A22:F22"/>
     <mergeCell ref="A25:F25"/>
-    <mergeCell ref="A80:F80"/>
-    <mergeCell ref="A81:F81"/>
     <mergeCell ref="A82:F82"/>
     <mergeCell ref="A83:F83"/>
     <mergeCell ref="A84:F84"/>
     <mergeCell ref="A85:F85"/>
     <mergeCell ref="A86:F86"/>
+    <mergeCell ref="A87:F87"/>
+    <mergeCell ref="A88:F88"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>